<commit_message>
fix(lib): update A.8.3 and bump version
</commit_message>
<xml_diff>
--- a/tools/excel/iso/iso42001-2023.xlsx
+++ b/tools/excel/iso/iso42001-2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abder/mydev/intuitem/staging/ciso-assistant-community/tools/excel/iso/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christopheb/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{772B7B8F-0352-8D4C-B93F-CBBCB43CBCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AB4970A-1317-F54C-93FB-00D37BFB83E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="-28020" windowWidth="50880" windowHeight="27860" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -809,9 +809,6 @@
     <t>External reporting</t>
   </si>
   <si>
-    <t>Report externally on AI system activities as required.</t>
-  </si>
-  <si>
     <t>A.8.4</t>
   </si>
   <si>
@@ -963,6 +960,9 @@
   </si>
   <si>
     <t>Controls</t>
+  </si>
+  <si>
+    <t>Enable relevant parties to report negative effects.</t>
   </si>
 </sst>
 </file>
@@ -1392,7 +1392,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1400,7 +1400,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="3">
-        <v>46006</v>
+        <v>46275</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -1513,7 +1513,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -1550,10 +1550,10 @@
     </row>
     <row r="10" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B10" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -1593,7 +1593,7 @@
         <v>11</v>
       </c>
       <c r="F1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1627,7 +1627,7 @@
         <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1647,7 +1647,7 @@
         <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -1667,7 +1667,7 @@
         <v>41</v>
       </c>
       <c r="F5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -1687,7 +1687,7 @@
         <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1721,7 +1721,7 @@
         <v>50</v>
       </c>
       <c r="F8" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -1741,7 +1741,7 @@
         <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -1761,7 +1761,7 @@
         <v>56</v>
       </c>
       <c r="F10" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1795,7 +1795,7 @@
         <v>62</v>
       </c>
       <c r="F12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -1815,7 +1815,7 @@
         <v>65</v>
       </c>
       <c r="F13" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1835,7 +1835,7 @@
         <v>68</v>
       </c>
       <c r="F14" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1869,7 +1869,7 @@
         <v>74</v>
       </c>
       <c r="F16" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -1889,7 +1889,7 @@
         <v>77</v>
       </c>
       <c r="F17" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -1909,7 +1909,7 @@
         <v>80</v>
       </c>
       <c r="F18" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -1929,7 +1929,7 @@
         <v>83</v>
       </c>
       <c r="F19" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1963,7 +1963,7 @@
         <v>89</v>
       </c>
       <c r="F21" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -1983,7 +1983,7 @@
         <v>92</v>
       </c>
       <c r="F22" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -2003,7 +2003,7 @@
         <v>95</v>
       </c>
       <c r="F23" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2037,7 +2037,7 @@
         <v>101</v>
       </c>
       <c r="F25" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -2057,7 +2057,7 @@
         <v>104</v>
       </c>
       <c r="F26" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -2077,7 +2077,7 @@
         <v>107</v>
       </c>
       <c r="F27" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -2097,7 +2097,7 @@
         <v>110</v>
       </c>
       <c r="F28" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2131,7 +2131,7 @@
         <v>116</v>
       </c>
       <c r="F30" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2165,7 +2165,7 @@
         <v>121</v>
       </c>
       <c r="F32" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -2185,7 +2185,7 @@
         <v>124</v>
       </c>
       <c r="F33" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2219,7 +2219,7 @@
         <v>129</v>
       </c>
       <c r="F35" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -2239,7 +2239,7 @@
         <v>132</v>
       </c>
       <c r="F36" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -2259,7 +2259,7 @@
         <v>135</v>
       </c>
       <c r="F37" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2293,7 +2293,7 @@
         <v>141</v>
       </c>
       <c r="F39" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -2313,7 +2313,7 @@
         <v>144</v>
       </c>
       <c r="F40" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2347,7 +2347,7 @@
         <v>149</v>
       </c>
       <c r="F42" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2367,7 +2367,7 @@
         <v>152</v>
       </c>
       <c r="F43" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2387,7 +2387,7 @@
         <v>155</v>
       </c>
       <c r="F44" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2421,7 +2421,7 @@
         <v>161</v>
       </c>
       <c r="F46" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2441,7 +2441,7 @@
         <v>164</v>
       </c>
       <c r="F47" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2475,7 +2475,7 @@
         <v>170</v>
       </c>
       <c r="F49" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2495,7 +2495,7 @@
         <v>173</v>
       </c>
       <c r="F50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2515,7 +2515,7 @@
         <v>176</v>
       </c>
       <c r="F51" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2535,7 +2535,7 @@
         <v>179</v>
       </c>
       <c r="F52" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2555,7 +2555,7 @@
         <v>182</v>
       </c>
       <c r="F53" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2589,7 +2589,7 @@
         <v>188</v>
       </c>
       <c r="F55" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2609,7 +2609,7 @@
         <v>191</v>
       </c>
       <c r="F56" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2629,7 +2629,7 @@
         <v>194</v>
       </c>
       <c r="F57" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2649,7 +2649,7 @@
         <v>197</v>
       </c>
       <c r="F58" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2697,7 +2697,7 @@
         <v>206</v>
       </c>
       <c r="F61" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2717,7 +2717,7 @@
         <v>209</v>
       </c>
       <c r="F62" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2751,7 +2751,7 @@
         <v>214</v>
       </c>
       <c r="F64" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2771,7 +2771,7 @@
         <v>217</v>
       </c>
       <c r="F65" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2791,7 +2791,7 @@
         <v>220</v>
       </c>
       <c r="F66" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2811,7 +2811,7 @@
         <v>223</v>
       </c>
       <c r="F67" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2831,7 +2831,7 @@
         <v>226</v>
       </c>
       <c r="F68" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2851,7 +2851,7 @@
         <v>229</v>
       </c>
       <c r="F69" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2871,7 +2871,7 @@
         <v>232</v>
       </c>
       <c r="F70" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2905,7 +2905,7 @@
         <v>238</v>
       </c>
       <c r="F72" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2925,7 +2925,7 @@
         <v>241</v>
       </c>
       <c r="F73" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2945,7 +2945,7 @@
         <v>244</v>
       </c>
       <c r="F74" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2965,7 +2965,7 @@
         <v>247</v>
       </c>
       <c r="F75" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2985,7 +2985,7 @@
         <v>250</v>
       </c>
       <c r="F76" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3019,7 +3019,7 @@
         <v>256</v>
       </c>
       <c r="F78" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3036,10 +3036,10 @@
         <v>258</v>
       </c>
       <c r="E79" t="s">
-        <v>259</v>
+        <v>310</v>
       </c>
       <c r="F79" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3050,16 +3050,16 @@
         <v>2</v>
       </c>
       <c r="C80" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="D80" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="D80" s="5" t="s">
+      <c r="E80" t="s">
         <v>261</v>
       </c>
-      <c r="E80" t="s">
-        <v>262</v>
-      </c>
       <c r="F80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3070,16 +3070,16 @@
         <v>2</v>
       </c>
       <c r="C81" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="D81" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="D81" s="5" t="s">
+      <c r="E81" t="s">
         <v>264</v>
       </c>
-      <c r="E81" t="s">
-        <v>265</v>
-      </c>
       <c r="F81" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3087,13 +3087,13 @@
         <v>1</v>
       </c>
       <c r="C82" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="D82" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="D82" s="5" t="s">
+      <c r="E82" t="s">
         <v>267</v>
-      </c>
-      <c r="E82" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3104,16 +3104,16 @@
         <v>2</v>
       </c>
       <c r="C83" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="D83" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="D83" s="5" t="s">
+      <c r="E83" t="s">
         <v>270</v>
       </c>
-      <c r="E83" t="s">
-        <v>271</v>
-      </c>
       <c r="F83" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3124,16 +3124,16 @@
         <v>2</v>
       </c>
       <c r="C84" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="D84" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="D84" s="5" t="s">
+      <c r="E84" t="s">
         <v>273</v>
       </c>
-      <c r="E84" t="s">
-        <v>274</v>
-      </c>
       <c r="F84" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="85" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3144,16 +3144,16 @@
         <v>2</v>
       </c>
       <c r="C85" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="D85" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="D85" s="5" t="s">
+      <c r="E85" t="s">
         <v>276</v>
       </c>
-      <c r="E85" t="s">
-        <v>277</v>
-      </c>
       <c r="F85" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="86" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3161,13 +3161,13 @@
         <v>1</v>
       </c>
       <c r="C86" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="D86" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="D86" s="5" t="s">
+      <c r="E86" t="s">
         <v>279</v>
-      </c>
-      <c r="E86" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="87" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3178,16 +3178,16 @@
         <v>2</v>
       </c>
       <c r="C87" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="D87" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="D87" s="5" t="s">
+      <c r="E87" t="s">
         <v>282</v>
       </c>
-      <c r="E87" t="s">
-        <v>283</v>
-      </c>
       <c r="F87" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="88" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3198,16 +3198,16 @@
         <v>2</v>
       </c>
       <c r="C88" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="D88" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="D88" s="5" t="s">
+      <c r="E88" t="s">
         <v>285</v>
       </c>
-      <c r="E88" t="s">
-        <v>286</v>
-      </c>
       <c r="F88" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3218,16 +3218,16 @@
         <v>2</v>
       </c>
       <c r="C89" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="D89" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="D89" s="5" t="s">
+      <c r="E89" t="s">
         <v>288</v>
       </c>
-      <c r="E89" t="s">
-        <v>289</v>
-      </c>
       <c r="F89" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -3280,7 +3280,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B1" t="s">
         <v>10</v>
@@ -3294,10 +3294,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C2" t="s">
         <v>291</v>
-      </c>
-      <c r="C2" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3305,10 +3305,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>292</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>293</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3316,10 +3316,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>294</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>295</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3327,10 +3327,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>296</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>297</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3338,10 +3338,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>298</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3349,10 +3349,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>300</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>301</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -3371,7 +3371,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -3379,7 +3379,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -3409,18 +3409,18 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(lib): clarify direction of external reporting on iso 42001:2023 (#4790)
* fix: clarify direction of external reporting

Initial wording is referring to provider -> user external reporting, while it's user -> provider

* fix version number and date

* fix(lib): update A.8.3 and bump version

---------

Co-authored-by: Abder <smimite@gmail.com>
</commit_message>
<xml_diff>
--- a/tools/excel/iso/iso42001-2023.xlsx
+++ b/tools/excel/iso/iso42001-2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abder/mydev/intuitem/staging/ciso-assistant-community/tools/excel/iso/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christopheb/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{772B7B8F-0352-8D4C-B93F-CBBCB43CBCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AB4970A-1317-F54C-93FB-00D37BFB83E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="-28020" windowWidth="50880" windowHeight="27860" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -809,9 +809,6 @@
     <t>External reporting</t>
   </si>
   <si>
-    <t>Report externally on AI system activities as required.</t>
-  </si>
-  <si>
     <t>A.8.4</t>
   </si>
   <si>
@@ -963,6 +960,9 @@
   </si>
   <si>
     <t>Controls</t>
+  </si>
+  <si>
+    <t>Enable relevant parties to report negative effects.</t>
   </si>
 </sst>
 </file>
@@ -1392,7 +1392,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1400,7 +1400,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="3">
-        <v>46006</v>
+        <v>46275</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -1513,7 +1513,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -1550,10 +1550,10 @@
     </row>
     <row r="10" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B10" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -1593,7 +1593,7 @@
         <v>11</v>
       </c>
       <c r="F1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1627,7 +1627,7 @@
         <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1647,7 +1647,7 @@
         <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -1667,7 +1667,7 @@
         <v>41</v>
       </c>
       <c r="F5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -1687,7 +1687,7 @@
         <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1721,7 +1721,7 @@
         <v>50</v>
       </c>
       <c r="F8" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -1741,7 +1741,7 @@
         <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -1761,7 +1761,7 @@
         <v>56</v>
       </c>
       <c r="F10" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1795,7 +1795,7 @@
         <v>62</v>
       </c>
       <c r="F12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -1815,7 +1815,7 @@
         <v>65</v>
       </c>
       <c r="F13" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1835,7 +1835,7 @@
         <v>68</v>
       </c>
       <c r="F14" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1869,7 +1869,7 @@
         <v>74</v>
       </c>
       <c r="F16" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -1889,7 +1889,7 @@
         <v>77</v>
       </c>
       <c r="F17" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -1909,7 +1909,7 @@
         <v>80</v>
       </c>
       <c r="F18" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -1929,7 +1929,7 @@
         <v>83</v>
       </c>
       <c r="F19" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1963,7 +1963,7 @@
         <v>89</v>
       </c>
       <c r="F21" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -1983,7 +1983,7 @@
         <v>92</v>
       </c>
       <c r="F22" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -2003,7 +2003,7 @@
         <v>95</v>
       </c>
       <c r="F23" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2037,7 +2037,7 @@
         <v>101</v>
       </c>
       <c r="F25" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -2057,7 +2057,7 @@
         <v>104</v>
       </c>
       <c r="F26" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -2077,7 +2077,7 @@
         <v>107</v>
       </c>
       <c r="F27" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -2097,7 +2097,7 @@
         <v>110</v>
       </c>
       <c r="F28" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2131,7 +2131,7 @@
         <v>116</v>
       </c>
       <c r="F30" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2165,7 +2165,7 @@
         <v>121</v>
       </c>
       <c r="F32" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -2185,7 +2185,7 @@
         <v>124</v>
       </c>
       <c r="F33" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2219,7 +2219,7 @@
         <v>129</v>
       </c>
       <c r="F35" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -2239,7 +2239,7 @@
         <v>132</v>
       </c>
       <c r="F36" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -2259,7 +2259,7 @@
         <v>135</v>
       </c>
       <c r="F37" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2293,7 +2293,7 @@
         <v>141</v>
       </c>
       <c r="F39" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -2313,7 +2313,7 @@
         <v>144</v>
       </c>
       <c r="F40" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2347,7 +2347,7 @@
         <v>149</v>
       </c>
       <c r="F42" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2367,7 +2367,7 @@
         <v>152</v>
       </c>
       <c r="F43" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2387,7 +2387,7 @@
         <v>155</v>
       </c>
       <c r="F44" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2421,7 +2421,7 @@
         <v>161</v>
       </c>
       <c r="F46" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2441,7 +2441,7 @@
         <v>164</v>
       </c>
       <c r="F47" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2475,7 +2475,7 @@
         <v>170</v>
       </c>
       <c r="F49" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2495,7 +2495,7 @@
         <v>173</v>
       </c>
       <c r="F50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2515,7 +2515,7 @@
         <v>176</v>
       </c>
       <c r="F51" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2535,7 +2535,7 @@
         <v>179</v>
       </c>
       <c r="F52" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2555,7 +2555,7 @@
         <v>182</v>
       </c>
       <c r="F53" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2589,7 +2589,7 @@
         <v>188</v>
       </c>
       <c r="F55" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2609,7 +2609,7 @@
         <v>191</v>
       </c>
       <c r="F56" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2629,7 +2629,7 @@
         <v>194</v>
       </c>
       <c r="F57" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2649,7 +2649,7 @@
         <v>197</v>
       </c>
       <c r="F58" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2697,7 +2697,7 @@
         <v>206</v>
       </c>
       <c r="F61" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2717,7 +2717,7 @@
         <v>209</v>
       </c>
       <c r="F62" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2751,7 +2751,7 @@
         <v>214</v>
       </c>
       <c r="F64" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2771,7 +2771,7 @@
         <v>217</v>
       </c>
       <c r="F65" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2791,7 +2791,7 @@
         <v>220</v>
       </c>
       <c r="F66" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2811,7 +2811,7 @@
         <v>223</v>
       </c>
       <c r="F67" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2831,7 +2831,7 @@
         <v>226</v>
       </c>
       <c r="F68" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2851,7 +2851,7 @@
         <v>229</v>
       </c>
       <c r="F69" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2871,7 +2871,7 @@
         <v>232</v>
       </c>
       <c r="F70" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2905,7 +2905,7 @@
         <v>238</v>
       </c>
       <c r="F72" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2925,7 +2925,7 @@
         <v>241</v>
       </c>
       <c r="F73" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2945,7 +2945,7 @@
         <v>244</v>
       </c>
       <c r="F74" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2965,7 +2965,7 @@
         <v>247</v>
       </c>
       <c r="F75" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2985,7 +2985,7 @@
         <v>250</v>
       </c>
       <c r="F76" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3019,7 +3019,7 @@
         <v>256</v>
       </c>
       <c r="F78" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3036,10 +3036,10 @@
         <v>258</v>
       </c>
       <c r="E79" t="s">
-        <v>259</v>
+        <v>310</v>
       </c>
       <c r="F79" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3050,16 +3050,16 @@
         <v>2</v>
       </c>
       <c r="C80" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="D80" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="D80" s="5" t="s">
+      <c r="E80" t="s">
         <v>261</v>
       </c>
-      <c r="E80" t="s">
-        <v>262</v>
-      </c>
       <c r="F80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3070,16 +3070,16 @@
         <v>2</v>
       </c>
       <c r="C81" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="D81" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="D81" s="5" t="s">
+      <c r="E81" t="s">
         <v>264</v>
       </c>
-      <c r="E81" t="s">
-        <v>265</v>
-      </c>
       <c r="F81" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3087,13 +3087,13 @@
         <v>1</v>
       </c>
       <c r="C82" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="D82" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="D82" s="5" t="s">
+      <c r="E82" t="s">
         <v>267</v>
-      </c>
-      <c r="E82" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3104,16 +3104,16 @@
         <v>2</v>
       </c>
       <c r="C83" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="D83" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="D83" s="5" t="s">
+      <c r="E83" t="s">
         <v>270</v>
       </c>
-      <c r="E83" t="s">
-        <v>271</v>
-      </c>
       <c r="F83" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3124,16 +3124,16 @@
         <v>2</v>
       </c>
       <c r="C84" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="D84" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="D84" s="5" t="s">
+      <c r="E84" t="s">
         <v>273</v>
       </c>
-      <c r="E84" t="s">
-        <v>274</v>
-      </c>
       <c r="F84" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="85" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3144,16 +3144,16 @@
         <v>2</v>
       </c>
       <c r="C85" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="D85" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="D85" s="5" t="s">
+      <c r="E85" t="s">
         <v>276</v>
       </c>
-      <c r="E85" t="s">
-        <v>277</v>
-      </c>
       <c r="F85" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="86" spans="1:6" ht="17" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3161,13 +3161,13 @@
         <v>1</v>
       </c>
       <c r="C86" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="D86" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="D86" s="5" t="s">
+      <c r="E86" t="s">
         <v>279</v>
-      </c>
-      <c r="E86" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="87" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3178,16 +3178,16 @@
         <v>2</v>
       </c>
       <c r="C87" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="D87" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="D87" s="5" t="s">
+      <c r="E87" t="s">
         <v>282</v>
       </c>
-      <c r="E87" t="s">
-        <v>283</v>
-      </c>
       <c r="F87" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="88" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3198,16 +3198,16 @@
         <v>2</v>
       </c>
       <c r="C88" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="D88" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="D88" s="5" t="s">
+      <c r="E88" t="s">
         <v>285</v>
       </c>
-      <c r="E88" t="s">
-        <v>286</v>
-      </c>
       <c r="F88" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3218,16 +3218,16 @@
         <v>2</v>
       </c>
       <c r="C89" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="D89" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="D89" s="5" t="s">
+      <c r="E89" t="s">
         <v>288</v>
       </c>
-      <c r="E89" t="s">
-        <v>289</v>
-      </c>
       <c r="F89" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -3280,7 +3280,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B1" t="s">
         <v>10</v>
@@ -3294,10 +3294,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C2" t="s">
         <v>291</v>
-      </c>
-      <c r="C2" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3305,10 +3305,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>292</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>293</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3316,10 +3316,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>294</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>295</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3327,10 +3327,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>296</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>297</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3338,10 +3338,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>298</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3349,10 +3349,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>300</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>301</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -3371,7 +3371,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -3379,7 +3379,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -3409,18 +3409,18 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>